<commit_message>
sync: 2026-05-21 10:58:24 from Cowork
</commit_message>
<xml_diff>
--- a/outputs/AI_Accounting_Margin_Model.xlsx
+++ b/outputs/AI_Accounting_Margin_Model.xlsx
@@ -261,7 +261,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="11"/>
   <chart>
     <title>
       <tx>
@@ -429,7 +428,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
   <chart>
     <title>
       <tx>
@@ -2227,15 +2225,15 @@
         <v/>
       </c>
       <c r="E24" s="11">
-        <f>E7*Inputs!E7</f>
+        <f>E8*Inputs!E7</f>
         <v/>
       </c>
       <c r="F24" s="11">
-        <f>F7*Inputs!E7</f>
+        <f>F8*Inputs!E7</f>
         <v/>
       </c>
       <c r="G24" s="11">
-        <f>G7*Inputs!E7</f>
+        <f>G8*Inputs!E7</f>
         <v/>
       </c>
     </row>
@@ -2255,15 +2253,15 @@
         <v/>
       </c>
       <c r="E25" s="11">
-        <f>E8*Inputs!E8</f>
+        <f>E9*Inputs!E8</f>
         <v/>
       </c>
       <c r="F25" s="11">
-        <f>F8*Inputs!E8</f>
+        <f>F9*Inputs!E8</f>
         <v/>
       </c>
       <c r="G25" s="11">
-        <f>G8*Inputs!E8</f>
+        <f>G9*Inputs!E8</f>
         <v/>
       </c>
     </row>
@@ -2283,15 +2281,15 @@
         <v/>
       </c>
       <c r="E26" s="11">
-        <f>E9*Inputs!E9</f>
+        <f>E10*Inputs!E9</f>
         <v/>
       </c>
       <c r="F26" s="11">
-        <f>F9*Inputs!E9</f>
+        <f>F10*Inputs!E9</f>
         <v/>
       </c>
       <c r="G26" s="11">
-        <f>G9*Inputs!E9</f>
+        <f>G10*Inputs!E9</f>
         <v/>
       </c>
     </row>
@@ -2311,15 +2309,15 @@
         <v/>
       </c>
       <c r="E27" s="11">
-        <f>E10*Inputs!E10</f>
+        <f>E11*Inputs!E10</f>
         <v/>
       </c>
       <c r="F27" s="11">
-        <f>F10*Inputs!E10</f>
+        <f>F11*Inputs!E10</f>
         <v/>
       </c>
       <c r="G27" s="11">
-        <f>G10*Inputs!E10</f>
+        <f>G11*Inputs!E10</f>
         <v/>
       </c>
     </row>
@@ -2339,15 +2337,15 @@
         <v/>
       </c>
       <c r="E28" s="11">
-        <f>E11*Inputs!E11</f>
+        <f>E12*Inputs!E11</f>
         <v/>
       </c>
       <c r="F28" s="11">
-        <f>F11*Inputs!E11</f>
+        <f>F12*Inputs!E11</f>
         <v/>
       </c>
       <c r="G28" s="11">
-        <f>G11*Inputs!E11</f>
+        <f>G12*Inputs!E11</f>
         <v/>
       </c>
     </row>

</xml_diff>